<commit_message>
Prune the tree and evaluation
</commit_message>
<xml_diff>
--- a/codebook.xlsx
+++ b/codebook.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Fall 2025\Data science\DataScience-Project-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02AB48AE-FAF7-49F6-88B4-40D0CD2444BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74E3E5F1-FCAE-481A-9FDB-2465A1214E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7ABD2A22-BBBF-413E-ACC5-9396B06F6957}"/>
   </bookViews>

</xml_diff>